<commit_message>
Lancement V1 : page d'accueil et conditions ouvertes à Google, prix sans TVA (autónomo non assujetti), NIF dans les mentions légales, prévisionnel refait sans TVA
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finance/WISHOP_previsionnel_2026-10.xlsx
+++ b/docs/finance/WISHOP_previsionnel_2026-10.xlsx
@@ -775,7 +775,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Guinée équatoriale (autónomo, à confirmer)</t>
+          <t>Guinée équatoriale (autónomo, non assujetti à la TVA)</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>4348</v>
+        <v>5000</v>
       </c>
       <c r="C55" s="6" t="n">
         <v>0.6</v>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>10870</v>
+        <v>12500</v>
       </c>
       <c r="C56" s="6" t="n">
         <v>0.3</v>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>21739</v>
+        <v>25000</v>
       </c>
       <c r="C57" s="6" t="n">
         <v>0.1</v>

</xml_diff>